<commit_message>
docs(ffxiv-global): add release date of 8.0 & add more videos
</commit_message>
<xml_diff>
--- a/blog/posts/ffxiv-global/expansion-packs.xlsx
+++ b/blog/posts/ffxiv-global/expansion-packs.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yilan Wang\Documents\GitHub\homepage\blog\posts\ffxiv-global\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Github\blog\blog\posts\ffxiv-global\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC04CB5C-FA2C-42F8-BB9B-7548839B9AA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC05A1D6-AF52-464F-B9F7-C7115D66927A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="资料片对比" sheetId="1" r:id="rId1"/>
@@ -267,10 +267,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>资料包</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>8.0 银海之天舟</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -499,10 +495,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>2027-01</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">8人大型
 </t>
@@ -637,6 +629,27 @@
   </si>
   <si>
     <t>阿卡狄亚登天斗技场</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>2027-0</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color theme="0"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>2-19</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>资料片</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -647,7 +660,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -796,6 +809,14 @@
       <color rgb="FFFFFFFF"/>
       <name val="思源宋体 Heavy"/>
       <family val="1"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="0"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
       <charset val="134"/>
     </font>
   </fonts>
@@ -1380,7 +1401,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="79.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>54</v>
+        <v>84</v>
       </c>
       <c r="B1" s="6" t="e" vm="1">
         <v>#VALUE!</v>
@@ -1425,12 +1446,12 @@
         <v>4</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:8" s="1" customFormat="1" ht="60" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B3" s="10">
         <v>41513</v>
@@ -1451,7 +1472,7 @@
         <v>45475</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:8" s="1" customFormat="1" ht="60" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1503,7 +1524,7 @@
         <v>12</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:8" s="1" customFormat="1" ht="60" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1511,25 +1532,25 @@
         <v>13</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E6" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="H6" s="13" t="s">
         <v>81</v>
-      </c>
-      <c r="F6" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="H6" s="13" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="1" customFormat="1" ht="60" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1542,7 +1563,7 @@
       </c>
       <c r="D7" s="14"/>
       <c r="E7" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F7" s="8" t="s">
         <v>16</v>
@@ -1557,7 +1578,7 @@
         <v>18</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>19</v>
@@ -1566,16 +1587,16 @@
         <v>20</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:8" s="1" customFormat="1" ht="60" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1595,7 +1616,7 @@
         <v>26</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>27</v>
@@ -1604,7 +1625,7 @@
     </row>
     <row r="10" spans="1:8" s="1" customFormat="1" ht="60" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B10" s="8" t="s">
         <v>28</v>
@@ -1616,21 +1637,21 @@
         <v>30</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>31</v>
       </c>
       <c r="G10" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="H10" s="8" t="s">
         <v>73</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:8" s="1" customFormat="1" ht="60" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>32</v>
@@ -1648,29 +1669,29 @@
         <v>36</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="1" customFormat="1" ht="60" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B12" s="14"/>
       <c r="C12" s="14"/>
       <c r="D12" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="E12" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="F12" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="G12" s="8" t="s">
         <v>68</v>
-      </c>
-      <c r="G12" s="8" t="s">
-        <v>69</v>
       </c>
       <c r="H12" s="8"/>
     </row>
@@ -1724,7 +1745,7 @@
       </c>
       <c r="B15" s="14"/>
       <c r="C15" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D15" s="8" t="s">
         <v>50</v>

</xml_diff>